<commit_message>
feat(reflector): complete 3-call verification chain — loading, ui-change, validity
</commit_message>
<xml_diff>
--- a/scenario.xlsx
+++ b/scenario.xlsx
@@ -2344,7 +2344,7 @@
       </c>
       <c r="J13" s="92" t="inlineStr">
         <is>
-          <t>3m 11s</t>
+          <t>2m 22s</t>
         </is>
       </c>
       <c r="K13" s="94" t="inlineStr">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="L13" s="95" t="inlineStr">
         <is>
-          <t>2026-05-29 22:01:48</t>
+          <t>2026-05-30 13:48:16</t>
         </is>
       </c>
       <c r="M13" s="96" t="inlineStr">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="N13" s="97" t="inlineStr">
         <is>
-          <t>outputs\predefined\NOTE-001_20260529_215813</t>
+          <t>outputs\predefined\NOTE-001_20260530_134524</t>
         </is>
       </c>
       <c r="O13" s="98" t="inlineStr">
@@ -2386,14 +2386,14 @@
       <c r="AA13" s="100" t="n"/>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>The live app screenshot clearly shows the home screen (beranda) of Xiaomi Notes after the user clicked the back button. The note titled "Rencana Skripsi 2026" is visible at the top of the list with the preview text "Selesaikan implementasi Multi-Agent Swarm untuk p..." and timestamp "22:00". This confirms the note has been successfully saved and is visible in the main list, satisfying the ultimate expected result: "Catatan tersimpan dan terlihat di daftar utama dengan judul 'Rencana Skripsi 2026</t>
+          <t>The live app screenshot shows the home screen (beranda) of Xiaomi Notes after the user clicked the back icon. The note "Rencana Skripsi 2026" is clearly visible at the top of the list with the preview text "Selesaikan implementasi Multi-Agent Swarm untuk p..." and timestamp "13:47". This confirms the note was successfully saved and is visible in the main list, which satisfies the ultimate expected result: "Catatan tersimpan dan terlihat di daftar utama dengan judul 'Rencana Skripsi 2026'".</t>
         </is>
       </c>
       <c r="AC13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AD13" t="n">
-        <v>39146</v>
+        <v>29616</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>

</xml_diff>